<commit_message>
Updated files Hardware testing
</commit_message>
<xml_diff>
--- a/Investigations/ADuM3190 Performance.xlsx
+++ b/Investigations/ADuM3190 Performance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\conor\Documents\College\Masters\Thesis\GeecPE2526\Investigations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{057BEC6B-8D0C-48E2-A3EA-5C55CA91A6D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D3EAC34-2EC7-4C0D-AB0D-FB0AB7BD7D71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{7CC224A8-521C-4B2A-9B71-E48C5C9E3FE3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7CC224A8-521C-4B2A-9B71-E48C5C9E3FE3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>